<commit_message>
Source GOV.UK year-one costs and make the parent link render.
Visa, IHS and London living now match the live GOV.UK pages, flights stay PLACEHOLDER, and the submission pack is ready to send.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/catalogue/task2-sources.xlsx
+++ b/data/catalogue/task2-sources.xlsx
@@ -692,7 +692,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Visa, IHS, London living, flights until Ambrosh / a sourced fare</t>
+          <t>Flights still PLACEHOLDER. Visa, IHS and London living sourced 2026-10-30.</t>
         </is>
       </c>
       <c r="D10" s="2" t="n"/>
@@ -737,7 +737,7 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Yellow cells on the GOV.UK tab are for Ambrosh: visa fee, IHS, and London living / maintenance, each with URL and date. Do not type invented numbers into the catalogue.</t>
+          <t>GOV.UK visa (£558), IHS (£776/year student) and London living (£13,761 visa financial requirement) were sourced 2026-10-30. Flights stay PLACEHOLDER. Yellow cells mean still missing. Do not invent a fare.</t>
         </is>
       </c>
       <c r="B14" s="2" t="n"/>
@@ -788,7 +788,7 @@
           <t>1. robots.txt — course/scholarship/India paths allowed; no login.
 2. Scrapy polite crawl (3s delay, 1 concurrent) into data/raw.
 3. Live check of UEL facts against the page (browser sample: Business Management BSc, Computer Science BSc, International Business Management MSc, scholarships, India).
-4. GOV.UK visa / IHS / living — Ambrosh.
+4. GOV.UK visa £558 / IHS £776 / London living £13,761 — sourced 2026-10-30.
 5. RBI INR/GBP reference from rbi.org.in, 1.00pm 28 Oct 2026, 126.4657 (FBIL).</t>
         </is>
       </c>
@@ -2118,13 +2118,11 @@
       </c>
       <c r="B2" s="9" t="inlineStr">
         <is>
-          <t>Ambrosh GOV.UK</t>
-        </is>
-      </c>
-      <c r="C2" s="12" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER</t>
-        </is>
+          <t>GOV.UK</t>
+        </is>
+      </c>
+      <c r="C2" s="10" t="n">
+        <v>13761</v>
       </c>
       <c r="D2" s="9" t="inlineStr">
         <is>
@@ -2133,12 +2131,12 @@
       </c>
       <c r="E2" s="9" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>Spot-check London living / maintenance.</t>
+          <t>Visa financial requirement £1,529 × 9 months. Not a personal spend forecast; not extra rent on halls.</t>
         </is>
       </c>
     </row>
@@ -2150,13 +2148,11 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Ambrosh GOV.UK</t>
-        </is>
-      </c>
-      <c r="C3" s="12" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER</t>
-        </is>
+          <t>GOV.UK</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="n">
+        <v>558</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
@@ -2165,12 +2161,12 @@
       </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>Spot-check student visa fee.</t>
+          <t>Student visa from outside the UK.</t>
         </is>
       </c>
     </row>
@@ -2182,27 +2178,25 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Ambrosh GOV.UK</t>
-        </is>
-      </c>
-      <c r="C4" s="12" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER</t>
-        </is>
+          <t>GOV.UK</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="n">
+        <v>776</v>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>https://www.gov.uk/healthcare-immigration-application</t>
+          <t>https://www.gov.uk/healthcare-immigration-application/how-much-pay</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>Spot-check Immigration Health Surcharge.</t>
+          <t>Student IHS rate per year. Year-one stack uses one year.</t>
         </is>
       </c>
     </row>
@@ -5566,7 +5560,7 @@
       </c>
       <c r="B107" s="9" t="inlineStr">
         <is>
-          <t>PLACEHOLDER</t>
+          <t>13761</t>
         </is>
       </c>
       <c r="C107" s="9" t="inlineStr">
@@ -5576,7 +5570,7 @@
       </c>
       <c r="D107" s="9" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E107" s="9" t="inlineStr">
@@ -5586,7 +5580,7 @@
       </c>
       <c r="F107" s="9" t="inlineStr">
         <is>
-          <t>Awaiting Ambrosh GOV.UK spot-check.</t>
+          <t>GOV.UK London financial requirement £1,529/month × 9 months. Visa maintenance figure, not a personal spend forecast. Do not add typical UEL room on top of this as a second rent.</t>
         </is>
       </c>
     </row>
@@ -5598,7 +5592,7 @@
       </c>
       <c r="B108" s="9" t="inlineStr">
         <is>
-          <t>PLACEHOLDER</t>
+          <t>558</t>
         </is>
       </c>
       <c r="C108" s="9" t="inlineStr">
@@ -5608,7 +5602,7 @@
       </c>
       <c r="D108" s="9" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E108" s="9" t="inlineStr">
@@ -5618,7 +5612,7 @@
       </c>
       <c r="F108" s="9" t="inlineStr">
         <is>
-          <t>Awaiting Ambrosh GOV.UK spot-check.</t>
+          <t>Student visa from outside the UK.</t>
         </is>
       </c>
     </row>
@@ -5630,17 +5624,17 @@
       </c>
       <c r="B109" s="9" t="inlineStr">
         <is>
-          <t>PLACEHOLDER</t>
+          <t>776</t>
         </is>
       </c>
       <c r="C109" s="9" t="inlineStr">
         <is>
-          <t>https://www.gov.uk/healthcare-immigration-application</t>
+          <t>https://www.gov.uk/healthcare-immigration-application/how-much-pay</t>
         </is>
       </c>
       <c r="D109" s="9" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E109" s="9" t="inlineStr">
@@ -5650,7 +5644,7 @@
       </c>
       <c r="F109" s="9" t="inlineStr">
         <is>
-          <t>Awaiting Ambrosh GOV.UK spot-check.</t>
+          <t>Student IHS rate per year. A longer visa costs more; year-one stack uses one year.</t>
         </is>
       </c>
     </row>
@@ -5801,7 +5795,7 @@
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="70" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -5834,69 +5828,75 @@
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>Student visa fee</t>
-        </is>
-      </c>
-      <c r="B2" s="12" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER</t>
-        </is>
-      </c>
-      <c r="C2" s="12" t="inlineStr">
+          <t>Student visa fee (from outside the UK)</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="n">
+        <v>558</v>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
         <is>
           <t>https://www.gov.uk/student-visa</t>
         </is>
       </c>
-      <c r="D2" s="12" t="inlineStr"/>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="E2" s="9" t="inlineStr">
         <is>
-          <t>Ambrosh</t>
+          <t>govuk-spot-check</t>
         </is>
       </c>
     </row>
     <row r="3" ht="36" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>Immigration Health Surcharge</t>
-        </is>
-      </c>
-      <c r="B3" s="12" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER</t>
-        </is>
-      </c>
-      <c r="C3" s="12" t="inlineStr">
-        <is>
-          <t>https://www.gov.uk/healthcare-immigration-application</t>
-        </is>
-      </c>
-      <c r="D3" s="12" t="inlineStr"/>
+          <t>Immigration Health Surcharge (student rate, one year)</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="n">
+        <v>776</v>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>https://www.gov.uk/healthcare-immigration-application/how-much-pay</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
-          <t>Ambrosh</t>
+          <t>govuk-spot-check</t>
         </is>
       </c>
     </row>
     <row r="4" ht="36" customHeight="1">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>London living / maintenance</t>
-        </is>
-      </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER</t>
-        </is>
-      </c>
-      <c r="C4" s="12" t="inlineStr">
+          <t>London living / maintenance (visa financial requirement, 9 months)</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="n">
+        <v>13761</v>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>https://www.gov.uk/student-visa/money</t>
         </is>
       </c>
-      <c r="D4" s="12" t="inlineStr"/>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>Ambrosh</t>
+          <t>govuk-spot-check</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
     <row r="6" ht="36" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>Paste the figure, the page URL, and the date you checked. Build will copy them into costs.json and sources.csv.</t>
+          <t>Living is the GOV.UK visa financial requirement, not a personal spend forecast. Do not add UEL halls on top of it as a second rent. Flights stay PLACEHOLDER.</t>
         </is>
       </c>
       <c r="B6" s="9" t="n"/>

</xml_diff>